<commit_message>
ops: verify October 28 feedback checks and both Excel deliveries before deadline
</commit_message>
<xml_diff>
--- a/work/2026-10-28臻肆工作台账.xlsx
+++ b/work/2026-10-28臻肆工作台账.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -480,10 +480,14 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>淘宝闪购差评申诉（每日11:20）</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
+          <t>负反馈列表申诉·双平台执行（每日08:30）</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-10-28T08:20:13</t>
+        </is>
+      </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
           <t>是</t>
@@ -491,23 +495,45 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>已随当日申诉完成</t>
+          <t>当日已完成</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>金鲨美团外卖差评申诉（每日14:25）</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
+          <t>负反馈列表申诉·双平台 Excel 汇总发群（每日08:30·申诉后即发）</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-10-28T08:21:20</t>
+        </is>
+      </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
+        <is>
+          <t>当日已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>淘宝闪购差评申诉（每日11:20）</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
         <is>
           <t>已随当日申诉完成</t>
         </is>
@@ -516,30 +542,48 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>应执行数量</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>已完成数量</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>2</v>
+          <t>金鲨美团外卖差评申诉（每日14:25）</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>已随当日申诉完成</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>应执行数量</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>已完成数量</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>汇总</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>未全绿-不发送</t>
         </is>

</xml_diff>

<commit_message>
ops: verify real merchant reseal and preserve negative analysis delivery evidence
</commit_message>
<xml_diff>
--- a/work/2026-10-28臻肆工作台账.xlsx
+++ b/work/2026-10-28臻肆工作台账.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -480,12 +480,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>负反馈列表申诉·双平台执行（每日08:30）</t>
+          <t>淘宝新增商家增量通知（每30分钟）</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-28T08:20:13</t>
+          <t>2026-10-28T08:30:39</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -502,12 +502,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>负反馈列表申诉·双平台 Excel 汇总发群（每日08:30·申诉后即发）</t>
+          <t>负反馈列表申诉·双平台执行（每日08:30）</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-28T08:21:20</t>
+          <t>2026-10-28T08:20:13</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -524,10 +524,14 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>淘宝闪购差评申诉（每日11:20）</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
+          <t>负反馈列表申诉·双平台 Excel 汇总发群（每日08:30·申诉后即发）</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-10-28T08:21:20</t>
+        </is>
+      </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
           <t>是</t>
@@ -535,14 +539,14 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>已随当日申诉完成</t>
+          <t>当日已完成</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>金鲨美团外卖差评申诉（每日14:25）</t>
+          <t>淘宝闪购差评申诉（每日11:20）</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -557,33 +561,51 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>应执行数量</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>24</v>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>金鲨美团外卖差评申诉（每日14:25）</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>已随当日申诉完成</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>已完成数量</t>
+          <t>应执行数量</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>已完成数量</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>汇总</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>未全绿-不发送</t>
         </is>

</xml_diff>

<commit_message>
ops: preserve final scheduled deliveries and image readback failure evidence
</commit_message>
<xml_diff>
--- a/work/2026-10-28臻肆工作台账.xlsx
+++ b/work/2026-10-28臻肆工作台账.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -485,7 +485,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-28T18:00:26</t>
+          <t>2026-10-28T18:30:22</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -714,14 +714,10 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>淘宝闪购自动差评申诉并企微反馈（每2小时·13:00起）</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>2026-10-28T17:05:37</t>
-        </is>
-      </c>
+          <t>金鲨美团外卖差评申诉（每日14:25）</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
       <c r="C15" s="3" t="inlineStr">
         <is>
           <t>是</t>
@@ -729,21 +725,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>当日已完成</t>
+          <t>已随当日申诉完成</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>金鲨美团外卖差评申诉（每日13:08）</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>2026-10-28T17:04:55</t>
-        </is>
-      </c>
+          <t>美团商家中心智能客服（15:00）</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
       <c r="C16" s="3" t="inlineStr">
         <is>
           <t>是</t>
@@ -751,17 +743,21 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>当日已完成</t>
+          <t>由当日末班覆盖</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>金鲨美团外卖差评申诉（每日14:25）</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
+          <t>美团商家中心智能客服（17:00·备发文档）</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-10-28T17:01:57</t>
+        </is>
+      </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
           <t>是</t>
@@ -769,45 +765,27 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>已随当日申诉完成</t>
+          <t>当日已完成</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>美团商家中心智能客服（15:00）</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
+          <t>淘宝闪购低优质商品的全部门店商品整改优化</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-10-28T17:14:04</t>
+        </is>
+      </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
-        <is>
-          <t>由当日末班覆盖</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>美团商家中心智能客服（17:00·备发文档）</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>2026-10-28T17:01:57</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
         <is>
           <t>当日已完成</t>
         </is>
@@ -816,52 +794,30 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>淘宝闪购低优质商品的全部门店商品整改优化</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>2026-10-28T17:14:04</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>当日已完成</t>
-        </is>
+          <t>应执行数量</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>已完成数量</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>应执行数量</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>已完成数量</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
           <t>汇总</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>未全绿-不发送</t>
         </is>

</xml_diff>